<commit_message>
Updated classes sheet and Dashboard
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="834">
   <si>
     <t>S.No.</t>
   </si>
@@ -2242,84 +2242,108 @@
     <t>Positive counterpart to TST_CLST_TC_22, which pairs a status and a label that match zero classes. TC_22 cannot distinguish AND from OR: if the filters were ORed, a zero-match pair would still return zero and TC_22 would still pass. This case is the only one that proves the AND. Added 2026-09-01 from the other team's TC_CLS_002, whose expected result states "Combined filters apply as an AND condition".</t>
   </si>
   <si>
+    <t>PASS. Combined filter (status Active + label A11y test) applied successfully; the page-level Clear link appeared, the 'Active classes (1)' heading updated, and exactly 1 matching class row (New Auto Test Class DND) was returned.</t>
+  </si>
+  <si>
+    <t>Automated — adminClassesTab.test.js (npm run P1AdminClassesTab_Thor, thor). Last run 2026-09-17: 24/24 passing.</t>
+  </si>
+  <si>
+    <t>Suite: adminClassesTab | 2026-09-17: Pass across 1 run</t>
+  </si>
+  <si>
+    <t>TST_GCAT_TC_11</t>
+  </si>
+  <si>
+    <t>Verify a grading category cannot be created with a name that already exists</t>
+  </si>
+  <si>
+    <t>#5 - Verify create grading category</t>
+  </si>
+  <si>
+    <t>On the Manage grading categories page, with at least one existing category whose name is known.</t>
+  </si>
+  <si>
+    <t>1. Note an existing category name and the current category count. 2. Click Create a grading category. 3. Enter the exact existing name. 4. Click Save. 5. Return to the list and re-count.</t>
+  </si>
+  <si>
+    <t>The name of a category already present in the school.</t>
+  </si>
+  <si>
+    <t>The duplicate name is not accepted: creation is blocked or warned per business rule, and the category count is unchanged. [ASSUMED] - the rule itself is unconfirmed; the other team's sheet also leaves it open ("handled per business rule").</t>
+  </si>
+  <si>
+    <t>Added 2026-09-01 from the other team's TC_CLS_005. We cover the empty name (TST_GCAT_TC_5) and the 50-character boundary (TST_GCAT_TC_3) but never re-use an existing name. Automation note: the GCAT suite deliberately generates names as AutoCat_create_&lt;epoch-ms&gt; to avoid collisions, so this case needs a fixed name plus a housekeeping step to remove it. Confirm the rule with the product owner before finalising the expected result - "blocked" and "warned but allowed" are different products.</t>
+  </si>
+  <si>
+    <t>PASS. Entering a duplicate category name disabled the Save button and displayed the inline validation message 'This name already exists'. The category count remained unchanged and the category name appeared exactly once in the list.</t>
+  </si>
+  <si>
+    <t>Automated as TST_GCAT_TC_11 in adminGradingCategories.test.js (npm run P1AdminGradingCategories_Thor). Verified live on thor (school FCN-CHZ-PDA). Resolved [ASSUMED] duplicate behavior.</t>
+  </si>
+  <si>
+    <t>Suite: adminGradingCategories | 2026-09-17: Pass across 2 runs</t>
+  </si>
+  <si>
+    <t>TST_GSCL_TC_15</t>
+  </si>
+  <si>
+    <t>Verify the Cambridge One default grading scale details page shows its classes list and notice but no bands section</t>
+  </si>
+  <si>
+    <t>#12 - Verify view details page of grading scale</t>
+  </si>
+  <si>
+    <t>On the Grading scales page. The system scale "Cambridge One grading scale" carries the default badge.</t>
+  </si>
+  <si>
+    <t>1. Open the Open drop down menu on "Cambridge One grading scale". 2. Click View details. 3. Read the page: heading, classes list, any notice, and whether a bands section is present.</t>
+  </si>
+  <si>
+    <t>The system scale "Cambridge One grading scale".</t>
+  </si>
+  <si>
+    <t>The details page shows the scale name, the linked Classes (n) list (or "No classes yet") and the pre-27-July-2023 notice. No "Grading scale bands" section is rendered, because the default scale's target varies by material. [ASSUMED] - the notice wording is not captured verbatim.</t>
+  </si>
+  <si>
+    <t>Added 2026-09-01 from the other team's TC_CLS_012, which opens both a custom scale and the default scale for comparison. Our TST_GSCL_TC_6 opens a custom scale only, and the default scale renders differently. The asymmetry is already recorded in this document's product reference and in TST_GSCL_TC_12's note - the case simply did not exist. Capture the notice text verbatim on the first live pass and clear the [ASSUMED].</t>
+  </si>
+  <si>
+    <t>PASS. The details page showed heading "Cambridge One grading scale", linked classes section heading "Classes (93)", and no "Grading scale bands" accordion section (element count 0).</t>
+  </si>
+  <si>
+    <t>Automated as TST_GSCL_TC_15 in adminGradingScales.test.js (npm run P1AdminGradingScales_Thor). Verified live on thor (school FCN-CHZ-PDA). Resolved [ASSUMED] notice/bands behavior.</t>
+  </si>
+  <si>
+    <t>Suite: adminGradingScales | 2026-09-17: Pass across 2 consecutive clean runs</t>
+  </si>
+  <si>
+    <t>TST_GSCL_TC_14</t>
+  </si>
+  <si>
+    <t>Verify a grading scale that is applied to a class cannot be deleted without warning</t>
+  </si>
+  <si>
+    <t>#15 - Verify deleting a grading scale</t>
+  </si>
+  <si>
+    <t>A non-default grading scale exists and is currently applied to at least one live class.</t>
+  </si>
+  <si>
+    <t>1. Apply a non-default scale to a class via Class grade settings. 2. Open the Grading scales page and that scale's Open drop down menu. 3. Click Delete. 4. Read the resulting dialog. 5. Cancel and confirm the scale is still listed and still applied to the class.</t>
+  </si>
+  <si>
+    <t>A non-default scale applied to &lt;CLASS_WITH_CUSTOM_SCALE&gt;.</t>
+  </si>
+  <si>
+    <t>Deletion of an in-use scale is prevented, or warns about the impact on the classes using it before proceeding, per business rule. The affected class(es) are identified to the admin. Cancelling leaves both the scale and the class assignment untouched. [ASSUMED] - behaviour and copy unconfirmed.</t>
+  </si>
+  <si>
+    <t>Added 2026-09-01 from the other team's TC_CLS_015_N1, which bundles two rules: the default scale and a scale in active use. Our TST_GSCL_TC_11 implements only the first. Suite placement: the precondition is a scale applied to a live class - the state the CGST suite already builds - so this case should run inside the CGST suite rather than the GSCL suite, exactly as TST_GSCL_TC_7 does.</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Blocked at design time (skill rule 4). TST_CLST_TC_4's Actual Result records that label VM1 matches no ACTIVE class on 3 July Test School 1. Unblock by applying an existing label to a known Active class on the target school, or by identifying a label/Active-class pair live; then ground the expected result and clear the [ASSUMED].</t>
-  </si>
-  <si>
-    <t>TST_GCAT_TC_10</t>
-  </si>
-  <si>
-    <t>Verify a grading category cannot be created with a name that already exists</t>
-  </si>
-  <si>
-    <t>#5 - Verify create grading category</t>
-  </si>
-  <si>
-    <t>On the Manage grading categories page, with at least one existing category whose name is known.</t>
-  </si>
-  <si>
-    <t>1. Note an existing category name and the current category count. 2. Click Create a grading category. 3. Enter the exact existing name. 4. Click Save. 5. Return to the list and re-count.</t>
-  </si>
-  <si>
-    <t>The name of a category already present in the school.</t>
-  </si>
-  <si>
-    <t>The duplicate name is not accepted: creation is blocked or warned per business rule, and the category count is unchanged. [ASSUMED] - the rule itself is unconfirmed; the other team's sheet also leaves it open ("handled per business rule").</t>
-  </si>
-  <si>
-    <t>Added 2026-09-01 from the other team's TC_CLS_005. We cover the empty name (TST_GCAT_TC_5) and the 50-character boundary (TST_GCAT_TC_3) but never re-use an existing name. Automation note: the GCAT suite deliberately generates names as AutoCat_create_&lt;epoch-ms&gt; to avoid collisions, so this case needs a fixed name plus a housekeeping step to remove it. Confirm the rule with the product owner before finalising the expected result - "blocked" and "warned but allowed" are different products.</t>
-  </si>
-  <si>
-    <t>TST_GSCL_TC_13</t>
-  </si>
-  <si>
-    <t>Verify the Cambridge One default grading scale details page shows its classes list and notice but no bands section</t>
-  </si>
-  <si>
-    <t>#12 - Verify view details page of grading scale</t>
-  </si>
-  <si>
-    <t>On the Grading scales page. The system scale "Cambridge One grading scale" carries the default badge.</t>
-  </si>
-  <si>
-    <t>1. Open the Open drop down menu on "Cambridge One grading scale". 2. Click View details. 3. Read the page: heading, classes list, any notice, and whether a bands section is present.</t>
-  </si>
-  <si>
-    <t>The system scale "Cambridge One grading scale".</t>
-  </si>
-  <si>
-    <t>The details page shows the scale name, the linked Classes (n) list (or "No classes yet") and the pre-27-July-2023 notice. No "Grading scale bands" section is rendered, because the default scale's target varies by material. [ASSUMED] - the notice wording is not captured verbatim.</t>
-  </si>
-  <si>
-    <t>Added 2026-09-01 from the other team's TC_CLS_012, which opens both a custom scale and the default scale for comparison. Our TST_GSCL_TC_6 opens a custom scale only, and the default scale renders differently. The asymmetry is already recorded in this document's product reference and in TST_GSCL_TC_12's note - the case simply did not exist. Capture the notice text verbatim on the first live pass and clear the [ASSUMED].</t>
-  </si>
-  <si>
-    <t>TST_GSCL_TC_14</t>
-  </si>
-  <si>
-    <t>Verify a grading scale that is applied to a class cannot be deleted without warning</t>
-  </si>
-  <si>
-    <t>#15 - Verify deleting a grading scale</t>
-  </si>
-  <si>
-    <t>A non-default grading scale exists and is currently applied to at least one live class.</t>
-  </si>
-  <si>
-    <t>1. Apply a non-default scale to a class via Class grade settings. 2. Open the Grading scales page and that scale's Open drop down menu. 3. Click Delete. 4. Read the resulting dialog. 5. Cancel and confirm the scale is still listed and still applied to the class.</t>
-  </si>
-  <si>
-    <t>A non-default scale applied to &lt;CLASS_WITH_CUSTOM_SCALE&gt;.</t>
-  </si>
-  <si>
-    <t>Deletion of an in-use scale is prevented, or warns about the impact on the classes using it before proceeding, per business rule. The affected class(es) are identified to the admin. Cancelling leaves both the scale and the class assignment untouched. [ASSUMED] - behaviour and copy unconfirmed.</t>
-  </si>
-  <si>
-    <t>Added 2026-09-01 from the other team's TC_CLS_015_N1, which bundles two rules: the default scale and a scale in active use. Our TST_GSCL_TC_11 implements only the first. Suite placement: the precondition is a scale applied to a live class - the state the CGST suite already builds - so this case should run inside the CGST suite rather than the GSCL suite, exactly as TST_GSCL_TC_7 does.</t>
-  </si>
-  <si>
     <t>TST_CGST_TC_7</t>
   </si>
   <si>
@@ -2344,7 +2368,7 @@
     <t>Added 2026-09-01 from the other team's TC_CLS_034, which covers weights, add and remove, and the 100% rule. Our TST_CGST_TC_3 only adds a category and TST_CGST_TC_6 only checks the 100% total, so removal was untested. Fits the existing CGST suite, which already creates and tears down its own class - no new fixture needed. Creates and mutates real data on that throwaway class.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_17</t>
+    <t>TST_CCLS_TC_24</t>
   </si>
   <si>
     <t>Verify the bulk Add teacher toolbar action applies the teacher to every selected class row</t>
@@ -2368,7 +2392,16 @@
     <t>Added 2026-09-01 from the other team's TC_CLS_036, which exercises the whole bulk toolbar. TST_BCCF_TC_9 covers bulk Start/End date only; its Remarks claim "the same pattern applies to bulk Add teacher / Add labels / Add Material" - a prose claim, not coverage. This case and TC_18-TC_21 turn that sentence into tests. Side-effect free - the form is not submitted.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_18</t>
+    <t>Teacher email applied to every selected row via bulk Add teacher toolbar action, and rows deselected after apply.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_24 (bulk suite). [ASSUMED] deselect-after-apply verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_24 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_25</t>
   </si>
   <si>
     <t>Verify the bulk Add Material toolbar action applies the material to every selected class row</t>
@@ -2389,7 +2422,16 @@
     <t>Added 2026-09-01 from TC_CLS_036 - see TST_BCCF_TC_17 Remarks. Side-effect free.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_19</t>
+    <t>Material applied to every selected row via bulk Add Material toolbar action, and rows deselected after apply.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_25 (bulk suite). [ASSUMED] deselect-after-apply verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_25 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_26</t>
   </si>
   <si>
     <t>Verify the bulk Add labels toolbar action applies the label to every selected class row</t>
@@ -2407,7 +2449,16 @@
     <t>Added 2026-09-01 from TC_CLS_036 - see TST_BCCF_TC_17 Remarks. Note TST_BCCF_TC_7 records that labels behave specially on Duplicate (an "Apply the labels to new classes too?" dialog); check whether the bulk label action raises anything similar. Side-effect free.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_20</t>
+    <t>Label applied to every selected row via bulk Add labels toolbar action, and rows deselected after apply.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_26 (bulk suite). [ASSUMED] deselect-after-apply verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_26 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_27</t>
   </si>
   <si>
     <t>Verify the bulk Show student progress toolbar action applies to every selected class row</t>
@@ -2425,7 +2476,16 @@
     <t>Added 2026-09-01 from TC_CLS_036. This is the toolbar control that produces a context class - the classes created this way are the subject of TST_CTXC_TC_1 and TST_CTXC_TC_2, so the two areas should be grounded in the same live pass. Side-effect free while the form is not submitted.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_21</t>
+    <t>Show student progress setting applied to selected rows via bulk toolbar action, confirming confirmation modal and applying setting across rows.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_27 (bulk suite). [ASSUMED] resolved live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_27 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_28</t>
   </si>
   <si>
     <t>Verify the bulk Remove toolbar action deletes exactly the selected class rows</t>
@@ -2444,6 +2504,15 @@
   </si>
   <si>
     <t>Added 2026-09-01 from TC_CLS_036. Deliberately leaves one row unselected: an action that removed all rows would still pass a case that only counted deletions. Side-effect free - the form is not submitted.</t>
+  </si>
+  <si>
+    <t>Exactly selected rows removed via bulk Remove toolbar action, confirmation dialog confirmed, Create N classes button count updated to remaining count, and unselected row survived.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_28 (bulk suite). [ASSUMED] confirmation dialog and surviving row verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_28 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
 </sst>
 </file>
@@ -6770,16 +6839,16 @@
         <v>743</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>249</v>
+        <v>28</v>
       </c>
       <c r="N84" s="3" t="s">
         <v>744</v>
       </c>
       <c r="O84" s="3" t="s">
-        <v>249</v>
+        <v>30</v>
       </c>
       <c r="P84" s="3" t="s">
-        <v>251</v>
+        <v>745</v>
       </c>
     </row>
     <row r="85" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6787,13 +6856,13 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>74</v>
@@ -6802,34 +6871,34 @@
         <v>54</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="K85" s="3" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="L85" s="3" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N85" s="3" t="s">
-        <v>743</v>
+        <v>755</v>
       </c>
       <c r="O85" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P85" s="3" t="s">
-        <v>220</v>
+        <v>756</v>
       </c>
     </row>
     <row r="86" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6837,13 +6906,13 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>20</v>
@@ -6852,34 +6921,34 @@
         <v>65</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="K86" s="3" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="L86" s="3" t="s">
-        <v>743</v>
+        <v>765</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N86" s="3" t="s">
-        <v>743</v>
+        <v>766</v>
       </c>
       <c r="O86" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P86" s="3" t="s">
-        <v>462</v>
+        <v>767</v>
       </c>
     </row>
     <row r="87" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6887,13 +6956,13 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>74</v>
@@ -6902,28 +6971,28 @@
         <v>54</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="K87" s="3" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="L87" s="3" t="s">
-        <v>743</v>
+        <v>776</v>
       </c>
       <c r="M87" s="3" t="s">
         <v>564</v>
       </c>
       <c r="N87" s="3" t="s">
-        <v>743</v>
+        <v>776</v>
       </c>
       <c r="O87" s="3" t="s">
         <v>338</v>
@@ -6937,13 +7006,13 @@
         <v>87</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>769</v>
+        <v>777</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>770</v>
+        <v>778</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>771</v>
+        <v>779</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>20</v>
@@ -6952,34 +7021,34 @@
         <v>54</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>773</v>
+        <v>781</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>774</v>
+        <v>782</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>775</v>
+        <v>783</v>
       </c>
       <c r="K88" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="L88" s="3" t="s">
         <v>776</v>
-      </c>
-      <c r="L88" s="3" t="s">
-        <v>743</v>
       </c>
       <c r="M88" s="3" t="s">
         <v>564</v>
       </c>
       <c r="N88" s="3" t="s">
-        <v>743</v>
+        <v>776</v>
       </c>
       <c r="O88" s="3" t="s">
-        <v>30</v>
+        <v>338</v>
       </c>
       <c r="P88" s="3" t="s">
-        <v>280</v>
+        <v>339</v>
       </c>
     </row>
     <row r="89" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6987,13 +7056,13 @@
         <v>88</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>778</v>
+        <v>786</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>20</v>
@@ -7002,34 +7071,34 @@
         <v>54</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>780</v>
+        <v>788</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>783</v>
+        <v>791</v>
       </c>
       <c r="K89" s="3" t="s">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="L89" s="3" t="s">
-        <v>743</v>
+        <v>793</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N89" s="3" t="s">
-        <v>743</v>
+        <v>794</v>
       </c>
       <c r="O89" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P89" s="3" t="s">
-        <v>339</v>
+        <v>795</v>
       </c>
     </row>
     <row r="90" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7037,13 +7106,13 @@
         <v>89</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>785</v>
+        <v>796</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>20</v>
@@ -7052,34 +7121,34 @@
         <v>54</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>788</v>
+        <v>799</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>789</v>
+        <v>800</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>790</v>
+        <v>801</v>
       </c>
       <c r="K90" s="3" t="s">
-        <v>791</v>
+        <v>802</v>
       </c>
       <c r="L90" s="3" t="s">
-        <v>743</v>
+        <v>803</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N90" s="3" t="s">
-        <v>743</v>
+        <v>804</v>
       </c>
       <c r="O90" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P90" s="3" t="s">
-        <v>339</v>
+        <v>805</v>
       </c>
     </row>
     <row r="91" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7087,13 +7156,13 @@
         <v>90</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>792</v>
+        <v>806</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>793</v>
+        <v>807</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>20</v>
@@ -7102,34 +7171,34 @@
         <v>54</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>794</v>
+        <v>808</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>795</v>
+        <v>809</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>796</v>
+        <v>810</v>
       </c>
       <c r="K91" s="3" t="s">
-        <v>797</v>
+        <v>811</v>
       </c>
       <c r="L91" s="3" t="s">
-        <v>743</v>
+        <v>812</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N91" s="3" t="s">
-        <v>743</v>
+        <v>813</v>
       </c>
       <c r="O91" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P91" s="3" t="s">
-        <v>339</v>
+        <v>814</v>
       </c>
     </row>
     <row r="92" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7137,13 +7206,13 @@
         <v>91</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>799</v>
+        <v>816</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>20</v>
@@ -7152,34 +7221,34 @@
         <v>54</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>800</v>
+        <v>817</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>801</v>
+        <v>818</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>802</v>
+        <v>819</v>
       </c>
       <c r="K92" s="3" t="s">
-        <v>803</v>
+        <v>820</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>743</v>
+        <v>821</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N92" s="3" t="s">
-        <v>743</v>
+        <v>822</v>
       </c>
       <c r="O92" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P92" s="3" t="s">
-        <v>339</v>
+        <v>823</v>
       </c>
     </row>
     <row r="93" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7187,13 +7256,13 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>804</v>
+        <v>824</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>805</v>
+        <v>825</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>20</v>
@@ -7202,34 +7271,34 @@
         <v>54</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>806</v>
+        <v>826</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>807</v>
+        <v>827</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>808</v>
+        <v>828</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>809</v>
+        <v>829</v>
       </c>
       <c r="K93" s="3" t="s">
-        <v>810</v>
+        <v>830</v>
       </c>
       <c r="L93" s="3" t="s">
-        <v>743</v>
+        <v>831</v>
       </c>
       <c r="M93" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N93" s="3" t="s">
-        <v>743</v>
+        <v>832</v>
       </c>
       <c r="O93" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P93" s="3" t="s">
-        <v>339</v>
+        <v>833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat/added missing classes testcases (#51)
* Implementation of TST_CLST_TC_24

* Implementation of TST_GCAT_TC_11

* Implementation of  TST_GSCL_TC_15

* Implementation of  TST_CCLS_TC_24  to TST_CCLS_TC_28

* Updated classes sheet and Dashboard
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="834">
   <si>
     <t>S.No.</t>
   </si>
@@ -2242,84 +2242,108 @@
     <t>Positive counterpart to TST_CLST_TC_22, which pairs a status and a label that match zero classes. TC_22 cannot distinguish AND from OR: if the filters were ORed, a zero-match pair would still return zero and TC_22 would still pass. This case is the only one that proves the AND. Added 2026-09-01 from the other team's TC_CLS_002, whose expected result states "Combined filters apply as an AND condition".</t>
   </si>
   <si>
+    <t>PASS. Combined filter (status Active + label A11y test) applied successfully; the page-level Clear link appeared, the 'Active classes (1)' heading updated, and exactly 1 matching class row (New Auto Test Class DND) was returned.</t>
+  </si>
+  <si>
+    <t>Automated — adminClassesTab.test.js (npm run P1AdminClassesTab_Thor, thor). Last run 2026-09-17: 24/24 passing.</t>
+  </si>
+  <si>
+    <t>Suite: adminClassesTab | 2026-09-17: Pass across 1 run</t>
+  </si>
+  <si>
+    <t>TST_GCAT_TC_11</t>
+  </si>
+  <si>
+    <t>Verify a grading category cannot be created with a name that already exists</t>
+  </si>
+  <si>
+    <t>#5 - Verify create grading category</t>
+  </si>
+  <si>
+    <t>On the Manage grading categories page, with at least one existing category whose name is known.</t>
+  </si>
+  <si>
+    <t>1. Note an existing category name and the current category count. 2. Click Create a grading category. 3. Enter the exact existing name. 4. Click Save. 5. Return to the list and re-count.</t>
+  </si>
+  <si>
+    <t>The name of a category already present in the school.</t>
+  </si>
+  <si>
+    <t>The duplicate name is not accepted: creation is blocked or warned per business rule, and the category count is unchanged. [ASSUMED] - the rule itself is unconfirmed; the other team's sheet also leaves it open ("handled per business rule").</t>
+  </si>
+  <si>
+    <t>Added 2026-09-01 from the other team's TC_CLS_005. We cover the empty name (TST_GCAT_TC_5) and the 50-character boundary (TST_GCAT_TC_3) but never re-use an existing name. Automation note: the GCAT suite deliberately generates names as AutoCat_create_&lt;epoch-ms&gt; to avoid collisions, so this case needs a fixed name plus a housekeeping step to remove it. Confirm the rule with the product owner before finalising the expected result - "blocked" and "warned but allowed" are different products.</t>
+  </si>
+  <si>
+    <t>PASS. Entering a duplicate category name disabled the Save button and displayed the inline validation message 'This name already exists'. The category count remained unchanged and the category name appeared exactly once in the list.</t>
+  </si>
+  <si>
+    <t>Automated as TST_GCAT_TC_11 in adminGradingCategories.test.js (npm run P1AdminGradingCategories_Thor). Verified live on thor (school FCN-CHZ-PDA). Resolved [ASSUMED] duplicate behavior.</t>
+  </si>
+  <si>
+    <t>Suite: adminGradingCategories | 2026-09-17: Pass across 2 runs</t>
+  </si>
+  <si>
+    <t>TST_GSCL_TC_15</t>
+  </si>
+  <si>
+    <t>Verify the Cambridge One default grading scale details page shows its classes list and notice but no bands section</t>
+  </si>
+  <si>
+    <t>#12 - Verify view details page of grading scale</t>
+  </si>
+  <si>
+    <t>On the Grading scales page. The system scale "Cambridge One grading scale" carries the default badge.</t>
+  </si>
+  <si>
+    <t>1. Open the Open drop down menu on "Cambridge One grading scale". 2. Click View details. 3. Read the page: heading, classes list, any notice, and whether a bands section is present.</t>
+  </si>
+  <si>
+    <t>The system scale "Cambridge One grading scale".</t>
+  </si>
+  <si>
+    <t>The details page shows the scale name, the linked Classes (n) list (or "No classes yet") and the pre-27-July-2023 notice. No "Grading scale bands" section is rendered, because the default scale's target varies by material. [ASSUMED] - the notice wording is not captured verbatim.</t>
+  </si>
+  <si>
+    <t>Added 2026-09-01 from the other team's TC_CLS_012, which opens both a custom scale and the default scale for comparison. Our TST_GSCL_TC_6 opens a custom scale only, and the default scale renders differently. The asymmetry is already recorded in this document's product reference and in TST_GSCL_TC_12's note - the case simply did not exist. Capture the notice text verbatim on the first live pass and clear the [ASSUMED].</t>
+  </si>
+  <si>
+    <t>PASS. The details page showed heading "Cambridge One grading scale", linked classes section heading "Classes (93)", and no "Grading scale bands" accordion section (element count 0).</t>
+  </si>
+  <si>
+    <t>Automated as TST_GSCL_TC_15 in adminGradingScales.test.js (npm run P1AdminGradingScales_Thor). Verified live on thor (school FCN-CHZ-PDA). Resolved [ASSUMED] notice/bands behavior.</t>
+  </si>
+  <si>
+    <t>Suite: adminGradingScales | 2026-09-17: Pass across 2 consecutive clean runs</t>
+  </si>
+  <si>
+    <t>TST_GSCL_TC_14</t>
+  </si>
+  <si>
+    <t>Verify a grading scale that is applied to a class cannot be deleted without warning</t>
+  </si>
+  <si>
+    <t>#15 - Verify deleting a grading scale</t>
+  </si>
+  <si>
+    <t>A non-default grading scale exists and is currently applied to at least one live class.</t>
+  </si>
+  <si>
+    <t>1. Apply a non-default scale to a class via Class grade settings. 2. Open the Grading scales page and that scale's Open drop down menu. 3. Click Delete. 4. Read the resulting dialog. 5. Cancel and confirm the scale is still listed and still applied to the class.</t>
+  </si>
+  <si>
+    <t>A non-default scale applied to &lt;CLASS_WITH_CUSTOM_SCALE&gt;.</t>
+  </si>
+  <si>
+    <t>Deletion of an in-use scale is prevented, or warns about the impact on the classes using it before proceeding, per business rule. The affected class(es) are identified to the admin. Cancelling leaves both the scale and the class assignment untouched. [ASSUMED] - behaviour and copy unconfirmed.</t>
+  </si>
+  <si>
+    <t>Added 2026-09-01 from the other team's TC_CLS_015_N1, which bundles two rules: the default scale and a scale in active use. Our TST_GSCL_TC_11 implements only the first. Suite placement: the precondition is a scale applied to a live class - the state the CGST suite already builds - so this case should run inside the CGST suite rather than the GSCL suite, exactly as TST_GSCL_TC_7 does.</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Blocked at design time (skill rule 4). TST_CLST_TC_4's Actual Result records that label VM1 matches no ACTIVE class on 3 July Test School 1. Unblock by applying an existing label to a known Active class on the target school, or by identifying a label/Active-class pair live; then ground the expected result and clear the [ASSUMED].</t>
-  </si>
-  <si>
-    <t>TST_GCAT_TC_10</t>
-  </si>
-  <si>
-    <t>Verify a grading category cannot be created with a name that already exists</t>
-  </si>
-  <si>
-    <t>#5 - Verify create grading category</t>
-  </si>
-  <si>
-    <t>On the Manage grading categories page, with at least one existing category whose name is known.</t>
-  </si>
-  <si>
-    <t>1. Note an existing category name and the current category count. 2. Click Create a grading category. 3. Enter the exact existing name. 4. Click Save. 5. Return to the list and re-count.</t>
-  </si>
-  <si>
-    <t>The name of a category already present in the school.</t>
-  </si>
-  <si>
-    <t>The duplicate name is not accepted: creation is blocked or warned per business rule, and the category count is unchanged. [ASSUMED] - the rule itself is unconfirmed; the other team's sheet also leaves it open ("handled per business rule").</t>
-  </si>
-  <si>
-    <t>Added 2026-09-01 from the other team's TC_CLS_005. We cover the empty name (TST_GCAT_TC_5) and the 50-character boundary (TST_GCAT_TC_3) but never re-use an existing name. Automation note: the GCAT suite deliberately generates names as AutoCat_create_&lt;epoch-ms&gt; to avoid collisions, so this case needs a fixed name plus a housekeeping step to remove it. Confirm the rule with the product owner before finalising the expected result - "blocked" and "warned but allowed" are different products.</t>
-  </si>
-  <si>
-    <t>TST_GSCL_TC_13</t>
-  </si>
-  <si>
-    <t>Verify the Cambridge One default grading scale details page shows its classes list and notice but no bands section</t>
-  </si>
-  <si>
-    <t>#12 - Verify view details page of grading scale</t>
-  </si>
-  <si>
-    <t>On the Grading scales page. The system scale "Cambridge One grading scale" carries the default badge.</t>
-  </si>
-  <si>
-    <t>1. Open the Open drop down menu on "Cambridge One grading scale". 2. Click View details. 3. Read the page: heading, classes list, any notice, and whether a bands section is present.</t>
-  </si>
-  <si>
-    <t>The system scale "Cambridge One grading scale".</t>
-  </si>
-  <si>
-    <t>The details page shows the scale name, the linked Classes (n) list (or "No classes yet") and the pre-27-July-2023 notice. No "Grading scale bands" section is rendered, because the default scale's target varies by material. [ASSUMED] - the notice wording is not captured verbatim.</t>
-  </si>
-  <si>
-    <t>Added 2026-09-01 from the other team's TC_CLS_012, which opens both a custom scale and the default scale for comparison. Our TST_GSCL_TC_6 opens a custom scale only, and the default scale renders differently. The asymmetry is already recorded in this document's product reference and in TST_GSCL_TC_12's note - the case simply did not exist. Capture the notice text verbatim on the first live pass and clear the [ASSUMED].</t>
-  </si>
-  <si>
-    <t>TST_GSCL_TC_14</t>
-  </si>
-  <si>
-    <t>Verify a grading scale that is applied to a class cannot be deleted without warning</t>
-  </si>
-  <si>
-    <t>#15 - Verify deleting a grading scale</t>
-  </si>
-  <si>
-    <t>A non-default grading scale exists and is currently applied to at least one live class.</t>
-  </si>
-  <si>
-    <t>1. Apply a non-default scale to a class via Class grade settings. 2. Open the Grading scales page and that scale's Open drop down menu. 3. Click Delete. 4. Read the resulting dialog. 5. Cancel and confirm the scale is still listed and still applied to the class.</t>
-  </si>
-  <si>
-    <t>A non-default scale applied to &lt;CLASS_WITH_CUSTOM_SCALE&gt;.</t>
-  </si>
-  <si>
-    <t>Deletion of an in-use scale is prevented, or warns about the impact on the classes using it before proceeding, per business rule. The affected class(es) are identified to the admin. Cancelling leaves both the scale and the class assignment untouched. [ASSUMED] - behaviour and copy unconfirmed.</t>
-  </si>
-  <si>
-    <t>Added 2026-09-01 from the other team's TC_CLS_015_N1, which bundles two rules: the default scale and a scale in active use. Our TST_GSCL_TC_11 implements only the first. Suite placement: the precondition is a scale applied to a live class - the state the CGST suite already builds - so this case should run inside the CGST suite rather than the GSCL suite, exactly as TST_GSCL_TC_7 does.</t>
-  </si>
-  <si>
     <t>TST_CGST_TC_7</t>
   </si>
   <si>
@@ -2344,7 +2368,7 @@
     <t>Added 2026-09-01 from the other team's TC_CLS_034, which covers weights, add and remove, and the 100% rule. Our TST_CGST_TC_3 only adds a category and TST_CGST_TC_6 only checks the 100% total, so removal was untested. Fits the existing CGST suite, which already creates and tears down its own class - no new fixture needed. Creates and mutates real data on that throwaway class.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_17</t>
+    <t>TST_CCLS_TC_24</t>
   </si>
   <si>
     <t>Verify the bulk Add teacher toolbar action applies the teacher to every selected class row</t>
@@ -2368,7 +2392,16 @@
     <t>Added 2026-09-01 from the other team's TC_CLS_036, which exercises the whole bulk toolbar. TST_BCCF_TC_9 covers bulk Start/End date only; its Remarks claim "the same pattern applies to bulk Add teacher / Add labels / Add Material" - a prose claim, not coverage. This case and TC_18-TC_21 turn that sentence into tests. Side-effect free - the form is not submitted.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_18</t>
+    <t>Teacher email applied to every selected row via bulk Add teacher toolbar action, and rows deselected after apply.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_24 (bulk suite). [ASSUMED] deselect-after-apply verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_24 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_25</t>
   </si>
   <si>
     <t>Verify the bulk Add Material toolbar action applies the material to every selected class row</t>
@@ -2389,7 +2422,16 @@
     <t>Added 2026-09-01 from TC_CLS_036 - see TST_BCCF_TC_17 Remarks. Side-effect free.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_19</t>
+    <t>Material applied to every selected row via bulk Add Material toolbar action, and rows deselected after apply.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_25 (bulk suite). [ASSUMED] deselect-after-apply verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_25 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_26</t>
   </si>
   <si>
     <t>Verify the bulk Add labels toolbar action applies the label to every selected class row</t>
@@ -2407,7 +2449,16 @@
     <t>Added 2026-09-01 from TC_CLS_036 - see TST_BCCF_TC_17 Remarks. Note TST_BCCF_TC_7 records that labels behave specially on Duplicate (an "Apply the labels to new classes too?" dialog); check whether the bulk label action raises anything similar. Side-effect free.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_20</t>
+    <t>Label applied to every selected row via bulk Add labels toolbar action, and rows deselected after apply.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_26 (bulk suite). [ASSUMED] deselect-after-apply verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_26 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_27</t>
   </si>
   <si>
     <t>Verify the bulk Show student progress toolbar action applies to every selected class row</t>
@@ -2425,7 +2476,16 @@
     <t>Added 2026-09-01 from TC_CLS_036. This is the toolbar control that produces a context class - the classes created this way are the subject of TST_CTXC_TC_1 and TST_CTXC_TC_2, so the two areas should be grounded in the same live pass. Side-effect free while the form is not submitted.</t>
   </si>
   <si>
-    <t>TST_BCCF_TC_21</t>
+    <t>Show student progress setting applied to selected rows via bulk toolbar action, confirming confirmation modal and applying setting across rows.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_27 (bulk suite). [ASSUMED] resolved live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_27 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
+  </si>
+  <si>
+    <t>TST_CCLS_TC_28</t>
   </si>
   <si>
     <t>Verify the bulk Remove toolbar action deletes exactly the selected class rows</t>
@@ -2444,6 +2504,15 @@
   </si>
   <si>
     <t>Added 2026-09-01 from TC_CLS_036. Deliberately leaves one row unselected: an action that removed all rows would still pass a case that only counted deletions. Side-effect free - the form is not submitted.</t>
+  </si>
+  <si>
+    <t>Exactly selected rows removed via bulk Remove toolbar action, confirmation dialog confirmed, Create N classes button count updated to remaining count, and unselected row survived.</t>
+  </si>
+  <si>
+    <t>Automated: TST_CCLS_TC_28 (bulk suite). [ASSUMED] confirmation dialog and surviving row verified live.</t>
+  </si>
+  <si>
+    <t>Automated as TST_CCLS_TC_28 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
 </sst>
 </file>
@@ -6770,16 +6839,16 @@
         <v>743</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>249</v>
+        <v>28</v>
       </c>
       <c r="N84" s="3" t="s">
         <v>744</v>
       </c>
       <c r="O84" s="3" t="s">
-        <v>249</v>
+        <v>30</v>
       </c>
       <c r="P84" s="3" t="s">
-        <v>251</v>
+        <v>745</v>
       </c>
     </row>
     <row r="85" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6787,13 +6856,13 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>74</v>
@@ -6802,34 +6871,34 @@
         <v>54</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="K85" s="3" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="L85" s="3" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N85" s="3" t="s">
-        <v>743</v>
+        <v>755</v>
       </c>
       <c r="O85" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P85" s="3" t="s">
-        <v>220</v>
+        <v>756</v>
       </c>
     </row>
     <row r="86" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6837,13 +6906,13 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>20</v>
@@ -6852,34 +6921,34 @@
         <v>65</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="K86" s="3" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="L86" s="3" t="s">
-        <v>743</v>
+        <v>765</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N86" s="3" t="s">
-        <v>743</v>
+        <v>766</v>
       </c>
       <c r="O86" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P86" s="3" t="s">
-        <v>462</v>
+        <v>767</v>
       </c>
     </row>
     <row r="87" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6887,13 +6956,13 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>74</v>
@@ -6902,28 +6971,28 @@
         <v>54</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="K87" s="3" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="L87" s="3" t="s">
-        <v>743</v>
+        <v>776</v>
       </c>
       <c r="M87" s="3" t="s">
         <v>564</v>
       </c>
       <c r="N87" s="3" t="s">
-        <v>743</v>
+        <v>776</v>
       </c>
       <c r="O87" s="3" t="s">
         <v>338</v>
@@ -6937,13 +7006,13 @@
         <v>87</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>769</v>
+        <v>777</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>770</v>
+        <v>778</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>771</v>
+        <v>779</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>20</v>
@@ -6952,34 +7021,34 @@
         <v>54</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>773</v>
+        <v>781</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>774</v>
+        <v>782</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>775</v>
+        <v>783</v>
       </c>
       <c r="K88" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="L88" s="3" t="s">
         <v>776</v>
-      </c>
-      <c r="L88" s="3" t="s">
-        <v>743</v>
       </c>
       <c r="M88" s="3" t="s">
         <v>564</v>
       </c>
       <c r="N88" s="3" t="s">
-        <v>743</v>
+        <v>776</v>
       </c>
       <c r="O88" s="3" t="s">
-        <v>30</v>
+        <v>338</v>
       </c>
       <c r="P88" s="3" t="s">
-        <v>280</v>
+        <v>339</v>
       </c>
     </row>
     <row r="89" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6987,13 +7056,13 @@
         <v>88</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>778</v>
+        <v>786</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>20</v>
@@ -7002,34 +7071,34 @@
         <v>54</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>780</v>
+        <v>788</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>783</v>
+        <v>791</v>
       </c>
       <c r="K89" s="3" t="s">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="L89" s="3" t="s">
-        <v>743</v>
+        <v>793</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N89" s="3" t="s">
-        <v>743</v>
+        <v>794</v>
       </c>
       <c r="O89" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P89" s="3" t="s">
-        <v>339</v>
+        <v>795</v>
       </c>
     </row>
     <row r="90" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7037,13 +7106,13 @@
         <v>89</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>785</v>
+        <v>796</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>20</v>
@@ -7052,34 +7121,34 @@
         <v>54</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>788</v>
+        <v>799</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>789</v>
+        <v>800</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>790</v>
+        <v>801</v>
       </c>
       <c r="K90" s="3" t="s">
-        <v>791</v>
+        <v>802</v>
       </c>
       <c r="L90" s="3" t="s">
-        <v>743</v>
+        <v>803</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N90" s="3" t="s">
-        <v>743</v>
+        <v>804</v>
       </c>
       <c r="O90" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P90" s="3" t="s">
-        <v>339</v>
+        <v>805</v>
       </c>
     </row>
     <row r="91" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7087,13 +7156,13 @@
         <v>90</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>792</v>
+        <v>806</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>793</v>
+        <v>807</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>20</v>
@@ -7102,34 +7171,34 @@
         <v>54</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>794</v>
+        <v>808</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>795</v>
+        <v>809</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>796</v>
+        <v>810</v>
       </c>
       <c r="K91" s="3" t="s">
-        <v>797</v>
+        <v>811</v>
       </c>
       <c r="L91" s="3" t="s">
-        <v>743</v>
+        <v>812</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N91" s="3" t="s">
-        <v>743</v>
+        <v>813</v>
       </c>
       <c r="O91" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P91" s="3" t="s">
-        <v>339</v>
+        <v>814</v>
       </c>
     </row>
     <row r="92" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7137,13 +7206,13 @@
         <v>91</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>799</v>
+        <v>816</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>20</v>
@@ -7152,34 +7221,34 @@
         <v>54</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>800</v>
+        <v>817</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>801</v>
+        <v>818</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>802</v>
+        <v>819</v>
       </c>
       <c r="K92" s="3" t="s">
-        <v>803</v>
+        <v>820</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>743</v>
+        <v>821</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N92" s="3" t="s">
-        <v>743</v>
+        <v>822</v>
       </c>
       <c r="O92" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P92" s="3" t="s">
-        <v>339</v>
+        <v>823</v>
       </c>
     </row>
     <row r="93" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -7187,13 +7256,13 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>804</v>
+        <v>824</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>805</v>
+        <v>825</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>20</v>
@@ -7202,34 +7271,34 @@
         <v>54</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>806</v>
+        <v>826</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>807</v>
+        <v>827</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>808</v>
+        <v>828</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>809</v>
+        <v>829</v>
       </c>
       <c r="K93" s="3" t="s">
-        <v>810</v>
+        <v>830</v>
       </c>
       <c r="L93" s="3" t="s">
-        <v>743</v>
+        <v>831</v>
       </c>
       <c r="M93" s="3" t="s">
-        <v>564</v>
+        <v>28</v>
       </c>
       <c r="N93" s="3" t="s">
-        <v>743</v>
+        <v>832</v>
       </c>
       <c r="O93" s="3" t="s">
-        <v>338</v>
+        <v>30</v>
       </c>
       <c r="P93" s="3" t="s">
-        <v>339</v>
+        <v>833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(manual): fix Classes id drift; restore evidence rows reset by registerSync
- Classes .xlsx rows 82-86: TST_CCLS_TC_24-28 -> TST_BCCF_TC_17-21, matching the .md
  (manual id; the CCLS id stays in Automation Evidence). The summary now shows the tool's counts:
  73 automated / 12 not.
- Students, Staff, Library, Reports, Generic: restore Status / Automation Status /
  Automation Evidence from the pre-removal archives. registerSync apply had run
  without archived audit runs and reset every evidence row to 'not executed'.
  The summary tables were recounted from the rows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
@@ -2194,7 +2194,7 @@
     <t>Added 2026-09-01 from the other team's TC_CLS_034, which covers weights, add and remove, and the 100% rule. Our TST_CGST_TC_3 only adds a category and TST_CGST_TC_6 only checks the 100% total, so removal was untested. Fits the existing CGST suite, which already creates and tears down its own class - no new fixture needed. Creates and mutates real data on that throwaway class.</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_24</t>
+    <t>TST_BCCF_TC_17</t>
   </si>
   <si>
     <t>Verify the bulk Add teacher toolbar action applies the teacher to every selected class row</t>
@@ -2227,7 +2227,7 @@
     <t>Automated as TST_CCLS_TC_24 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_25</t>
+    <t>TST_BCCF_TC_18</t>
   </si>
   <si>
     <t>Verify the bulk Add Material toolbar action applies the material to every selected class row</t>
@@ -2257,7 +2257,7 @@
     <t>Automated as TST_CCLS_TC_25 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_26</t>
+    <t>TST_BCCF_TC_19</t>
   </si>
   <si>
     <t>Verify the bulk Add labels toolbar action applies the label to every selected class row</t>
@@ -2284,7 +2284,7 @@
     <t>Automated as TST_CCLS_TC_26 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_27</t>
+    <t>TST_BCCF_TC_20</t>
   </si>
   <si>
     <t>Verify the bulk Show student progress toolbar action applies to every selected class row</t>
@@ -2311,7 +2311,7 @@
     <t>Automated as TST_CCLS_TC_27 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_28</t>
+    <t>TST_BCCF_TC_21</t>
   </si>
   <si>
     <t>Verify the bulk Remove toolbar action deletes exactly the selected class rows</t>

</xml_diff>

<commit_message>
test(manual): fix Classes id drift; restore evidence rows reset by registerSync (#57)
- Classes .xlsx rows 82-86: TST_CCLS_TC_24-28 -> TST_BCCF_TC_17-21, matching the .md
  (manual id; the CCLS id stays in Automation Evidence). The summary now shows the tool's counts:
  73 automated / 12 not.
- Students, Staff, Library, Reports, Generic: restore Status / Automation Status /
  Automation Evidence from the pre-removal archives. registerSync apply had run
  without archived audit runs and reset every evidence row to 'not executed'.
  The summary tables were recounted from the rows.

Co-authored-by: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
@@ -2194,7 +2194,7 @@
     <t>Added 2026-09-01 from the other team's TC_CLS_034, which covers weights, add and remove, and the 100% rule. Our TST_CGST_TC_3 only adds a category and TST_CGST_TC_6 only checks the 100% total, so removal was untested. Fits the existing CGST suite, which already creates and tears down its own class - no new fixture needed. Creates and mutates real data on that throwaway class.</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_24</t>
+    <t>TST_BCCF_TC_17</t>
   </si>
   <si>
     <t>Verify the bulk Add teacher toolbar action applies the teacher to every selected class row</t>
@@ -2227,7 +2227,7 @@
     <t>Automated as TST_CCLS_TC_24 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_25</t>
+    <t>TST_BCCF_TC_18</t>
   </si>
   <si>
     <t>Verify the bulk Add Material toolbar action applies the material to every selected class row</t>
@@ -2257,7 +2257,7 @@
     <t>Automated as TST_CCLS_TC_25 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_26</t>
+    <t>TST_BCCF_TC_19</t>
   </si>
   <si>
     <t>Verify the bulk Add labels toolbar action applies the label to every selected class row</t>
@@ -2284,7 +2284,7 @@
     <t>Automated as TST_CCLS_TC_26 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_27</t>
+    <t>TST_BCCF_TC_20</t>
   </si>
   <si>
     <t>Verify the bulk Show student progress toolbar action applies to every selected class row</t>
@@ -2311,7 +2311,7 @@
     <t>Automated as TST_CCLS_TC_27 | Suite: schoolAdminAddClassBulk | 2026-09-17: Pass</t>
   </si>
   <si>
-    <t>TST_CCLS_TC_28</t>
+    <t>TST_BCCF_TC_21</t>
   </si>
   <si>
     <t>Verify the bulk Remove toolbar action deletes exactly the selected class rows</t>

</xml_diff>